<commit_message>
refactor: name map variants charge and battery
</commit_message>
<xml_diff>
--- a/projects/map/02-BOM/map-BOM.xlsx
+++ b/projects/map/02-BOM/map-BOM.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1 充电版" sheetId="1" r:id="R5d1f73bf4cea48b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v2 电池版" sheetId="2" r:id="R7e5271ba03c34fee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="charge 充电版" sheetId="1" r:id="Rb3211a4043114af4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="battery 电池版" sheetId="2" r:id="R54e371812f484981"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -418,7 +418,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>map v1 充电版 · 物料表</x:v>
+        <x:v>map charge 充电版 · 物料表</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -1067,7 +1067,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R217bc0ddcd9d434c"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R922a441cd1cb421f"/>
 </x:worksheet>
 </file>
 
@@ -1093,7 +1093,7 @@
     </x:row>
     <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>map v2 电池版 · 物料表</x:v>
+        <x:v>map battery 电池版 · 物料表</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -1584,6 +1584,6 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd505f905bd574913"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a3c7630b8c943ef"/>
 </x:worksheet>
 </file>
</xml_diff>